<commit_message>
03.05.2025 - Yeni form əlavə olundu
</commit_message>
<xml_diff>
--- a/Fayllar/Muhasibat/Yanasmalar/LCR hesabat yanasmalari.xlsx
+++ b/Fayllar/Muhasibat/Yanasmalar/LCR hesabat yanasmalari.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="94">
   <si>
     <t>c15</t>
   </si>
@@ -285,9 +285,6 @@
     <t>14010+14030</t>
   </si>
   <si>
-    <t>90 gune qeder gecikmeler hamisi+90 den artiq olanlar hesabat ayinda olanlarin meblegi</t>
-  </si>
-  <si>
     <t>qiymetli kag novbeti ayin tarixine uygun gelenleri</t>
   </si>
   <si>
@@ -302,12 +299,18 @@
   <si>
     <t>04-03-2024 den sonra Vuqar deysdirdi</t>
   </si>
+  <si>
+    <t>90 gune qeder gecikmesi olanlarin ayliq odenisi+90 gunden artiq olanlarin 6 ayda odediyi meblegin 6 ayliq ortalamasi</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +342,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -360,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -371,6 +382,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -50272,63 +50284,66 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="80.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="107" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="52.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="G1" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -50336,23 +50351,23 @@
         <v>15770</v>
       </c>
       <c r="C10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" t="s">
         <v>91</v>
       </c>
-      <c r="D10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>41</v>
       </c>
@@ -50360,26 +50375,26 @@
         <v>86</v>
       </c>
       <c r="C13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" t="s">
         <v>88</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>89</v>
       </c>
-      <c r="E13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>44</v>
       </c>

</xml_diff>